<commit_message>
docs: split KEYMAP grid between col 6 and 7; add README
- tools/KUKEY42.layout.json: move the right-inner center column from x=6
  to x=7 so the doc generator's split gap falls between displayed columns
  6 and 7 (true 6+6 split). Left-inner keys now render in col 6, right-inner
  in col 7, matching the physical board. Regenerated KEYMAP.html/.xlsx.
- README.md: new, linking KEYMAP.html (relative + htmlpreview) and the
  custom-behavior naming convention.

https://claude.ai/code/session_011NPTsK3j5KN481k1Zjtvqa
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -548,8 +548,8 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
@@ -600,12 +600,12 @@
           <t>6</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>8</t>
@@ -1014,13 +1014,13 @@
 &amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>N
@@ -1088,12 +1088,12 @@
           <t>L7</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>L7</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -1156,12 +1156,12 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
           <t>〃</t>
@@ -1230,13 +1230,13 @@
 &amp;mo SYMBOL</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;mo VIM_NORMAL_1</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -1289,12 +1289,12 @@
           <t>L1</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>L2</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr">
         <is>
           <t>ENTER</t>
@@ -1345,12 +1345,12 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
           <t>L1</t>
@@ -1747,13 +1747,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr"/>
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="7" t="inlineStr">
         <is>
           <t>N
@@ -1907,13 +1907,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;mo VIM_NORMAL_2</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -1958,12 +1958,12 @@
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr"/>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr"/>
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr"/>
@@ -1998,12 +1998,12 @@
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr"/>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr"/>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="9" t="inlineStr"/>
       <c r="L27" s="9" t="inlineStr"/>
@@ -2591,13 +2591,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="7" t="inlineStr">
         <is>
           <t>N
@@ -2761,13 +2761,13 @@
 &amp;mo VIM_NORMAL_2</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -3146,13 +3146,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr"/>
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr"/>
       <c r="J51" s="7" t="inlineStr">
         <is>
           <t>N
@@ -3254,13 +3254,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr"/>
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr"/>
       <c r="J53" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -3551,13 +3551,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr"/>
+      <c r="I60" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr"/>
       <c r="J60" s="7" t="inlineStr">
         <is>
           <t>N
@@ -3651,13 +3651,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr"/>
+      <c r="I62" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I62" s="7" t="inlineStr"/>
       <c r="J62" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -3936,13 +3936,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H69" s="7" t="inlineStr">
+      <c r="H69" s="7" t="inlineStr"/>
+      <c r="I69" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I69" s="7" t="inlineStr"/>
       <c r="J69" s="7" t="inlineStr">
         <is>
           <t>N
@@ -4036,13 +4036,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="7" t="inlineStr"/>
+      <c r="I71" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -4361,13 +4361,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H78" s="7" t="inlineStr">
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I78" s="7" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr">
         <is>
           <t>N
@@ -4461,13 +4461,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr"/>
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I80" s="7" t="inlineStr"/>
       <c r="J80" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -4746,13 +4746,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H87" s="7" t="inlineStr">
+      <c r="H87" s="7" t="inlineStr"/>
+      <c r="I87" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I87" s="7" t="inlineStr"/>
       <c r="J87" s="7" t="inlineStr">
         <is>
           <t>N
@@ -4846,13 +4846,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H89" s="7" t="inlineStr">
+      <c r="H89" s="7" t="inlineStr"/>
+      <c r="I89" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I89" s="7" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -5289,13 +5289,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H98" s="7" t="inlineStr">
+      <c r="H98" s="7" t="inlineStr"/>
+      <c r="I98" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I98" s="7" t="inlineStr"/>
       <c r="J98" s="7" t="inlineStr">
         <is>
           <t>N
@@ -5419,13 +5419,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H100" s="7" t="inlineStr">
+      <c r="H100" s="7" t="inlineStr"/>
+      <c r="I100" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I100" s="7" t="inlineStr"/>
       <c r="J100" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -5494,8 +5494,8 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
@@ -5546,12 +5546,12 @@
           <t>6</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>8</t>
@@ -5960,13 +5960,13 @@
 &amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>N
@@ -6034,12 +6034,12 @@
           <t>&amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>&amp;mo BLUETOOTH</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr">
         <is>
           <t>&amp;kp N</t>
@@ -6102,12 +6102,12 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
           <t>〃</t>
@@ -6176,13 +6176,13 @@
 &amp;mo SYMBOL</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;mo VIM_NORMAL_1</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -6235,12 +6235,12 @@
           <t>&amp;mo SYMBOL</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>&amp;mo VIM_NORMAL_1</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr">
         <is>
           <t>&amp;lt SYMBOL ENTER</t>
@@ -6291,12 +6291,12 @@
           <t>〃</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
           <t>&amp;lt SYMBOL ENTER</t>
@@ -6693,13 +6693,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr"/>
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="7" t="inlineStr">
         <is>
           <t>N
@@ -6853,13 +6853,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;mo VIM_NORMAL_2</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -6904,12 +6904,12 @@
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr"/>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr"/>
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>&amp;mo VIM_NORMAL_2</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr"/>
@@ -6944,12 +6944,12 @@
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr"/>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>〃</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr"/>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>〃</t>
+        </is>
+      </c>
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="9" t="inlineStr"/>
       <c r="L27" s="9" t="inlineStr"/>
@@ -7571,13 +7571,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="7" t="inlineStr">
         <is>
           <t>N
@@ -7742,13 +7742,13 @@
 &amp;mo VIM_NORMAL_2</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr"/>
+      <c r="I42" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -8139,13 +8139,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr"/>
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr"/>
       <c r="J51" s="7" t="inlineStr">
         <is>
           <t>N
@@ -8247,13 +8247,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr"/>
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr"/>
       <c r="J53" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -8544,13 +8544,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H60" s="7" t="inlineStr"/>
+      <c r="I60" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr"/>
       <c r="J60" s="7" t="inlineStr">
         <is>
           <t>N
@@ -8644,13 +8644,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr"/>
+      <c r="I62" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I62" s="7" t="inlineStr"/>
       <c r="J62" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -8937,13 +8937,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H69" s="7" t="inlineStr">
+      <c r="H69" s="7" t="inlineStr"/>
+      <c r="I69" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I69" s="7" t="inlineStr"/>
       <c r="J69" s="7" t="inlineStr">
         <is>
           <t>N
@@ -9045,13 +9045,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="7" t="inlineStr"/>
+      <c r="I71" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -9378,13 +9378,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H78" s="7" t="inlineStr">
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I78" s="7" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr">
         <is>
           <t>N
@@ -9486,13 +9486,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr"/>
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I80" s="7" t="inlineStr"/>
       <c r="J80" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -9799,13 +9799,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H87" s="7" t="inlineStr">
+      <c r="H87" s="7" t="inlineStr"/>
+      <c r="I87" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I87" s="7" t="inlineStr"/>
       <c r="J87" s="7" t="inlineStr">
         <is>
           <t>N
@@ -9907,13 +9907,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H89" s="7" t="inlineStr">
+      <c r="H89" s="7" t="inlineStr"/>
+      <c r="I89" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I89" s="7" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
@@ -10349,13 +10349,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H98" s="7" t="inlineStr">
+      <c r="H98" s="7" t="inlineStr"/>
+      <c r="I98" s="7" t="inlineStr">
         <is>
           <t>mo中央R
 &amp;none</t>
         </is>
       </c>
-      <c r="I98" s="7" t="inlineStr"/>
       <c r="J98" s="7" t="inlineStr">
         <is>
           <t>N
@@ -10473,13 +10473,13 @@
 &amp;none</t>
         </is>
       </c>
-      <c r="H100" s="7" t="inlineStr">
+      <c r="H100" s="7" t="inlineStr"/>
+      <c r="I100" s="7" t="inlineStr">
         <is>
           <t>mo2 (center)
 &amp;none</t>
         </is>
       </c>
-      <c r="I100" s="7" t="inlineStr"/>
       <c r="J100" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER

</xml_diff>